<commit_message>
pushing missed files from framework
</commit_message>
<xml_diff>
--- a/excel/login-test-cases.xlsx
+++ b/excel/login-test-cases.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3155" uniqueCount="905">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3276" uniqueCount="971">
   <si>
     <t>Bugasura - test case pack</t>
   </si>
@@ -2946,6 +2946,374 @@
     <t>#critical_bugs_moving contains "Rate at Which Critical Issues are Closed"; #issues_update_container contains "Line Chart : Getting flat line for Weekly and monthly periodicities in the rendered line chart and also displaying wrong data points using Summation operator in Device Data source."; 635838 is not ticked; 635838 is ticked</t>
   </si>
   <si>
+    <t>TC_LOGIN_141</t>
+  </si>
+  <si>
+    <t>#tr_1751001 &gt; .tabulator-cell.tabulator-cell--checkbox &gt; .rounded-checkbox-cont &gt; .rounded-checkbox-ui — #ap_notifications_panel contains "Notification Preferences"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open https://my.bugasura.io/
+Enter the email
+Enter the password
+Click Sign In
+Click Notifications
+Click Notification settings
+Click .ba-switch__track
+Untick Enable Notifications Enable
+Click .ba-switch__thumb
+Tick Enable Notifications Enable
+Click Close
+Click Faclon labs
+Click #tr_635838 &gt; .tabulator-cell.tabulator-cell--checkbox &gt; .rounded-checkbox-cont &gt; .rounded-checkbox-ui
+Click Requirements Management
+Click Manage
+Click Test Data Test Data
+Click Notifications Notifications
+Click Home
+Click iosense.io
+Click #tr_1751001 &gt; .tabulator-cell.tabulator-cell--checkbox &gt; .rounded-checkbox-cont &gt; .rounded-checkbox-ui</t>
+  </si>
+  <si>
+    <t>#ap_notifications_panel contains "Notification Preferences"; #requirements_banner contains "Requirements management need not be hard"; #show_all_teams contains "Sravya D"; heading contains "Team work"; #main-content contains "Customize Data Sets"; #main-content contains "Not one more tool"; Enable Notifications Receive notifications for activity acro is ticked; Enable Notifications Receive notifications for activity acro is not ticked; 1751002 is not ticked; 1751001 is ticked</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_142</t>
+  </si>
+  <si>
+    <t>Notifications Notifications — #requirements_banner contains "Requirements management need not be hard"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open https://my.bugasura.io/
+Enter the email
+Enter the password
+Click Sign In
+Click Faclon labs
+Click #tr_635838 &gt; .tabulator-cell.tabulator-cell--checkbox &gt; .rounded-checkbox-cont &gt; .rounded-checkbox-ui
+Click Requirements Management
+Click Notifications
+Click Notification settings
+Click Close
+Click Manage
+Click Test Data Test Data
+Click Notifications Notifications</t>
+  </si>
+  <si>
+    <t>#requirements_banner contains "Requirements management need not be hard"; #show_all_teams contains "Sravya D"; heading contains "Team work"; #main-content contains "Customize Data Sets"; #main-content contains "Not one more tool"; 635838 is ticked; Enable Notifications Receive notifications for activity acro is ticked</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_143</t>
+  </si>
+  <si>
+    <t>Close — heading contains "A comprehensive visual overview of bug status, trends, and metrics for effective monitoring and analysis."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open https://my.bugasura.io/
+Enter the email
+Enter the password
+Click Sign In
+Click Faclon labs
+Click #tr_635838 &gt; .tabulator-cell.tabulator-cell--checkbox &gt; .rounded-checkbox-cont &gt; .rounded-checkbox-ui
+Click Reports
+Click Activity
+Click Notifications
+Click Notification settings
+Click .ba-switch__thumb
+Untick Enable Notifications Enable
+Click .ba-switch__track
+Tick Enable Notifications Enable
+Click Close</t>
+  </si>
+  <si>
+    <t>Heading contains "A comprehensive visual overview of bug status, trends, and metrics for effective monitoring and analysis."; heading contains "Activity"; 635838 is ticked; Enable Notifications Receive notifications for activity acro is ticked; Enable Notifications Receive notifications for activity acro is not ticked</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_144</t>
+  </si>
+  <si>
+    <t>#tr_1751001 &gt; .tabulator-cell.tabulator-cell--checkbox &gt; .rounded-checkbox-cont &gt; .rounded-checkbox-ui — #show_all_teams contains "Sravya D"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open https://my.bugasura.io/
+Enter the email
+Enter the password
+Click Sign In
+Click Manage
+Click Test Data Test Data
+Click Notifications
+Click Notification settings
+Click .ba-switch__thumb
+Untick Enable Notifications Enable
+Click Enable Notifications Enable
+Untick Enable Notifications Enable
+Click Close
+Click Home
+Click Faclon labs
+Click #tr_635838 &gt; .tabulator-cell.tabulator-cell--checkbox &gt; .rounded-checkbox-cont &gt; .rounded-checkbox-ui
+Click Home
+Click iosense.io
+Click .rounded-checkbox-ui
+Click #tr_1751001 &gt; .tabulator-cell.tabulator-cell--checkbox &gt; .rounded-checkbox-cont &gt; .rounded-checkbox-ui</t>
+  </si>
+  <si>
+    <t>#show_all_teams contains "Sravya D"; #show_all_teams contains "Naresh Kumaar"; heading contains "Team work"; #main-content contains "Customize Data Sets"; Enable Notifications Receive notifications for activity acro is ticked; 1751002 is ticked</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_145</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open https://my.bugasura.io/
+Enter the email
+Enter the password
+Click Sign In
+Click Faclon labs
+Click #tr_638416 &gt; .tabulator-cell.tabulator-cell--checkbox &gt; .rounded-checkbox-cont &gt; .rounded-checkbox-ui
+Click .rounded-checkbox-ui</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_146</t>
+  </si>
+  <si>
+    <t>Home — #all_apps contains "Faclon labs"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open https://my.bugasura.io/
+Enter the email
+Click Password
+Enter the password
+Click Sign In
+Click + Create Project
+Click Enter a Project Name
+Enter the enter a project name
+Click Select your team 
+Click Faclon
+Click Desktop Web
+Click Create Project
+Click Home</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Email = maneeswar.reddy@moolya.com
+Password = &lt;valid-password&gt;
+Enter a Project Name = Test7</t>
+  </si>
+  <si>
+    <t>#all_apps contains "Faclon labs"</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_147</t>
+  </si>
+  <si>
+    <t>Create Project — #main-content contains "Test1"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open https://my.bugasura.io/
+Enter the email
+Enter the password
+Click Sign In
+Click + Create Project
+Click Enter a Project Name
+Enter the enter a project name
+Click Select your team 
+Click Faclon
+Click Desktop Web
+Click Create Project</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Email = maneeswar.reddy@moolya.com
+Password = &lt;valid-password&gt;
+Enter a Project Name = Test1</t>
+  </si>
+  <si>
+    <t>#main-content contains "Test1"</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_148</t>
+  </si>
+  <si>
+    <t>+ Create Project</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open https://my.bugasura.io/
+Enter the email
+Click Password
+Enter the password
+Click Sign In
+Click + Create Project
+Click Enter a Project Name
+Enter the enter a project name
+Click Select your team 
+Click Faclon
+Click Desktop Web
+Click Cancel
+Click + Create Project</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Email = maneeswar.reddy@moolya.com
+Password = &lt;valid-password&gt;
+Enter a Project Name = Test3</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_149</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open https://my.bugasura.io/
+Enter the email
+Enter the password
+Click Sign In
+Click + Create Project
+Click Enter a Project Name
+Enter the enter a project name
+Click Select your team 
+Click Faclon
+Click Desktop Web
+Click Cancel
+Click + Create Project
+Click Cancel</t>
+  </si>
+  <si>
+    <t>#first_report_modal contains "Create New Project"; h2 contains "All Projects"</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_150</t>
+  </si>
+  <si>
+    <t>+ Create Project — #first_report_modal contains "Create New Project"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open https://my.bugasura.io/
+Enter the email
+Enter the password
+Click Sign In
+Click + Create Project
+Click Enter a Project Name
+Enter the enter a project name
+Click Select your team 
+Click Faclon
+Click Desktop Web
+Click button
+Click + Create Project</t>
+  </si>
+  <si>
+    <t>#first_report_modal contains "Create New Project"</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_151</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open https://my.bugasura.io/
+Enter the email
+Enter the password
+Click Sign In
+Click + Create Project
+Click Cancel
+Click + Create Project</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_152</t>
+  </si>
+  <si>
+    <t>Following — #bug_report_multi_search contains "0"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open https://my.bugasura.io/
+Enter the email
+Click Password
+Enter the password
+Click Sign In
+Click Filter Filter 
+Click Android
+Click Filter Filter 
+Click Filter Filter 
+Click Following</t>
+  </si>
+  <si>
+    <t>#bug_report_multi_search contains "0"; #bug_report_multi_search contains "Android"</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_153</t>
+  </si>
+  <si>
+    <t>Team Projects — #all_apps contains "Faclon labs"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open https://my.bugasura.io/
+Enter the email
+Enter the password
+Click Sign In
+Click Filter Filter 
+Click Faclon
+Click  Faclon
+Click kwysight
+Click Team Projects</t>
+  </si>
+  <si>
+    <t>#all_apps contains "Faclon labs"; #all_apps contains "sample"; h2 contains "Team Projects"</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_154</t>
+  </si>
+  <si>
+    <t>Drafts (3)  — Draft is visible</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open https://my.bugasura.io/
+Enter the email
+Enter the password
+Click Sign In
+Click Faclon labs
+Click #tr_636432 &gt; .tabulator-cell.tabulator-cell--checkbox &gt; .rounded-checkbox-cont &gt; .rounded-checkbox-ui
+Click .rounded-checkbox-ui
+Click Drafts (3) </t>
+  </si>
+  <si>
+    <t>Draft is visible</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_155</t>
+  </si>
+  <si>
+    <t>Search — #all_apps contains "Faclon labs"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open https://my.bugasura.io/
+Enter the email
+Click Password
+Enter the password
+Click Sign In
+Click Search
+Enter the search
+Press Enter in Search</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Email = maneeswar.reddy@moolya.com
+Password = &lt;valid-password&gt;
+Search = Faclon</t>
+  </si>
+  <si>
+    <t>#all_apps contains "Faclon labs"; input is visible</t>
+  </si>
+  <si>
+    <t>TC_LOGIN_156</t>
+  </si>
+  <si>
+    <t>Activity — #tc_update_status_1755479 contains "New"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open https://my.bugasura.io/
+Enter the email
+Click Password
+Enter the password
+Click Sign In
+Click Faclon labs
+Click .rounded-checkbox-ui
+Click #tr_636432 &gt; .tabulator-cell.tabulator-cell--checkbox &gt; .rounded-checkbox-cont &gt; .rounded-checkbox-ui
+Click .panel.panel-body.new-counts &gt; .u-dis-f-rc
+Click Reports
+Click Activity</t>
+  </si>
+  <si>
+    <t>#tc_update_status_1755479 contains "New"; heading contains "A comprehensive visual overview of bug status, trends, and metrics for effective monitoring and analysis."; heading contains "Activity"; 1755479 is not ticked; 1755479 is ticked; 636432 is ticked</t>
+  </si>
+  <si>
     <t>TC_PROJ_001</t>
   </si>
   <si>
@@ -3856,6 +4224,25 @@
   </si>
   <si>
     <t>#critical_bugs_moving contains "Rate at Which Critical Issues are Closed"; heading contains "Activity"; 635838 is not ticked; 635838 is ticked</t>
+  </si>
+  <si>
+    <t>TC_DASHBOARD_028</t>
+  </si>
+  <si>
+    <t>Reports — heading contains "A comprehensive visual overview of bug status, trends, and metrics for effective monitoring and analysis."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open https://my.bugasura.io/
+Enter the email
+Enter the password
+Click Sign In
+Click Faclon labs
+Click .rounded-checkbox-ui
+Click #tr_636432 &gt; .tabulator-cell.tabulator-cell--checkbox &gt; .rounded-checkbox-cont &gt; .rounded-checkbox-ui
+Click Reports</t>
+  </si>
+  <si>
+    <t>Heading contains "A comprehensive visual overview of bug status, trends, and metrics for effective monitoring and analysis."; 1755479 is not ticked; 1755479 is ticked; 636432 is ticked</t>
   </si>
 </sst>
 </file>
@@ -4418,7 +4805,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AG134"/>
+  <dimension ref="A1:AG150"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -12742,6 +13129,598 @@
       <c r="AE134" s="8"/>
       <c r="AF134" s="8"/>
       <c r="AG134" s="8"/>
+    </row>
+    <row r="135" spans="1:33" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A135" s="8" t="s">
+        <v>674</v>
+      </c>
+      <c r="B135" s="8"/>
+      <c r="C135" s="8"/>
+      <c r="D135" s="8" t="s">
+        <v>675</v>
+      </c>
+      <c r="E135" s="8"/>
+      <c r="F135" s="8"/>
+      <c r="G135" s="8" t="s">
+        <v>676</v>
+      </c>
+      <c r="H135" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="I135" s="8" t="s">
+        <v>677</v>
+      </c>
+      <c r="J135" s="8"/>
+      <c r="K135" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="N135" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y135" s="8"/>
+      <c r="Z135" s="8"/>
+      <c r="AA135" s="8"/>
+      <c r="AB135" s="8"/>
+      <c r="AC135" s="8"/>
+      <c r="AD135" s="8"/>
+      <c r="AE135" s="8"/>
+      <c r="AF135" s="8"/>
+      <c r="AG135" s="8"/>
+    </row>
+    <row r="136" spans="1:33" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A136" s="8" t="s">
+        <v>678</v>
+      </c>
+      <c r="B136" s="8"/>
+      <c r="C136" s="8"/>
+      <c r="D136" s="8" t="s">
+        <v>679</v>
+      </c>
+      <c r="E136" s="8"/>
+      <c r="F136" s="8"/>
+      <c r="G136" s="8" t="s">
+        <v>680</v>
+      </c>
+      <c r="H136" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="I136" s="8" t="s">
+        <v>681</v>
+      </c>
+      <c r="J136" s="8"/>
+      <c r="K136" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="N136" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y136" s="8"/>
+      <c r="Z136" s="8"/>
+      <c r="AA136" s="8"/>
+      <c r="AB136" s="8"/>
+      <c r="AC136" s="8"/>
+      <c r="AD136" s="8"/>
+      <c r="AE136" s="8"/>
+      <c r="AF136" s="8"/>
+      <c r="AG136" s="8"/>
+    </row>
+    <row r="137" spans="1:33" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A137" s="8" t="s">
+        <v>682</v>
+      </c>
+      <c r="B137" s="8"/>
+      <c r="C137" s="8"/>
+      <c r="D137" s="8" t="s">
+        <v>683</v>
+      </c>
+      <c r="E137" s="8"/>
+      <c r="F137" s="8"/>
+      <c r="G137" s="8" t="s">
+        <v>684</v>
+      </c>
+      <c r="H137" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="I137" s="8" t="s">
+        <v>685</v>
+      </c>
+      <c r="J137" s="8"/>
+      <c r="K137" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="N137" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y137" s="8"/>
+      <c r="Z137" s="8"/>
+      <c r="AA137" s="8"/>
+      <c r="AB137" s="8"/>
+      <c r="AC137" s="8"/>
+      <c r="AD137" s="8"/>
+      <c r="AE137" s="8"/>
+      <c r="AF137" s="8"/>
+      <c r="AG137" s="8"/>
+    </row>
+    <row r="138" spans="1:33" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A138" s="8" t="s">
+        <v>686</v>
+      </c>
+      <c r="B138" s="8"/>
+      <c r="C138" s="8"/>
+      <c r="D138" s="8" t="s">
+        <v>687</v>
+      </c>
+      <c r="E138" s="8"/>
+      <c r="F138" s="8"/>
+      <c r="G138" s="8" t="s">
+        <v>688</v>
+      </c>
+      <c r="H138" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="I138" s="8" t="s">
+        <v>689</v>
+      </c>
+      <c r="J138" s="8"/>
+      <c r="K138" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="N138" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y138" s="8"/>
+      <c r="Z138" s="8"/>
+      <c r="AA138" s="8"/>
+      <c r="AB138" s="8"/>
+      <c r="AC138" s="8"/>
+      <c r="AD138" s="8"/>
+      <c r="AE138" s="8"/>
+      <c r="AF138" s="8"/>
+      <c r="AG138" s="8"/>
+    </row>
+    <row r="139" spans="1:33" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A139" s="8" t="s">
+        <v>690</v>
+      </c>
+      <c r="B139" s="8"/>
+      <c r="C139" s="8"/>
+      <c r="D139" s="8" t="s">
+        <v>444</v>
+      </c>
+      <c r="E139" s="8"/>
+      <c r="F139" s="8"/>
+      <c r="G139" s="8" t="s">
+        <v>691</v>
+      </c>
+      <c r="H139" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="I139" s="8" t="s">
+        <v>453</v>
+      </c>
+      <c r="J139" s="8"/>
+      <c r="K139" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="N139" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y139" s="8"/>
+      <c r="Z139" s="8"/>
+      <c r="AA139" s="8"/>
+      <c r="AB139" s="8"/>
+      <c r="AC139" s="8"/>
+      <c r="AD139" s="8"/>
+      <c r="AE139" s="8"/>
+      <c r="AF139" s="8"/>
+      <c r="AG139" s="8"/>
+    </row>
+    <row r="140" spans="1:33" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A140" s="8" t="s">
+        <v>692</v>
+      </c>
+      <c r="B140" s="8"/>
+      <c r="C140" s="8"/>
+      <c r="D140" s="8" t="s">
+        <v>693</v>
+      </c>
+      <c r="E140" s="8"/>
+      <c r="F140" s="8"/>
+      <c r="G140" s="8" t="s">
+        <v>694</v>
+      </c>
+      <c r="H140" s="8" t="s">
+        <v>695</v>
+      </c>
+      <c r="I140" s="8" t="s">
+        <v>696</v>
+      </c>
+      <c r="J140" s="8"/>
+      <c r="K140" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="N140" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y140" s="8"/>
+      <c r="Z140" s="8"/>
+      <c r="AA140" s="8"/>
+      <c r="AB140" s="8"/>
+      <c r="AC140" s="8"/>
+      <c r="AD140" s="8"/>
+      <c r="AE140" s="8"/>
+      <c r="AF140" s="8"/>
+      <c r="AG140" s="8"/>
+    </row>
+    <row r="141" spans="1:33" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A141" s="8" t="s">
+        <v>697</v>
+      </c>
+      <c r="B141" s="8"/>
+      <c r="C141" s="8"/>
+      <c r="D141" s="8" t="s">
+        <v>698</v>
+      </c>
+      <c r="E141" s="8"/>
+      <c r="F141" s="8"/>
+      <c r="G141" s="8" t="s">
+        <v>699</v>
+      </c>
+      <c r="H141" s="8" t="s">
+        <v>700</v>
+      </c>
+      <c r="I141" s="8" t="s">
+        <v>701</v>
+      </c>
+      <c r="J141" s="8"/>
+      <c r="K141" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="N141" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y141" s="8"/>
+      <c r="Z141" s="8"/>
+      <c r="AA141" s="8"/>
+      <c r="AB141" s="8"/>
+      <c r="AC141" s="8"/>
+      <c r="AD141" s="8"/>
+      <c r="AE141" s="8"/>
+      <c r="AF141" s="8"/>
+      <c r="AG141" s="8"/>
+    </row>
+    <row r="142" spans="1:33" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A142" s="8" t="s">
+        <v>702</v>
+      </c>
+      <c r="B142" s="8"/>
+      <c r="C142" s="8"/>
+      <c r="D142" s="8" t="s">
+        <v>703</v>
+      </c>
+      <c r="E142" s="8"/>
+      <c r="F142" s="8"/>
+      <c r="G142" s="8" t="s">
+        <v>704</v>
+      </c>
+      <c r="H142" s="8" t="s">
+        <v>705</v>
+      </c>
+      <c r="I142" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="J142" s="8"/>
+      <c r="K142" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="N142" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y142" s="8"/>
+      <c r="Z142" s="8"/>
+      <c r="AA142" s="8"/>
+      <c r="AB142" s="8"/>
+      <c r="AC142" s="8"/>
+      <c r="AD142" s="8"/>
+      <c r="AE142" s="8"/>
+      <c r="AF142" s="8"/>
+      <c r="AG142" s="8"/>
+    </row>
+    <row r="143" spans="1:33" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A143" s="8" t="s">
+        <v>706</v>
+      </c>
+      <c r="B143" s="8"/>
+      <c r="C143" s="8"/>
+      <c r="D143" s="8" t="s">
+        <v>200</v>
+      </c>
+      <c r="E143" s="8"/>
+      <c r="F143" s="8"/>
+      <c r="G143" s="8" t="s">
+        <v>707</v>
+      </c>
+      <c r="H143" s="8" t="s">
+        <v>705</v>
+      </c>
+      <c r="I143" s="8" t="s">
+        <v>708</v>
+      </c>
+      <c r="J143" s="8"/>
+      <c r="K143" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="N143" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y143" s="8"/>
+      <c r="Z143" s="8"/>
+      <c r="AA143" s="8"/>
+      <c r="AB143" s="8"/>
+      <c r="AC143" s="8"/>
+      <c r="AD143" s="8"/>
+      <c r="AE143" s="8"/>
+      <c r="AF143" s="8"/>
+      <c r="AG143" s="8"/>
+    </row>
+    <row r="144" spans="1:33" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A144" s="8" t="s">
+        <v>709</v>
+      </c>
+      <c r="B144" s="8"/>
+      <c r="C144" s="8"/>
+      <c r="D144" s="8" t="s">
+        <v>710</v>
+      </c>
+      <c r="E144" s="8"/>
+      <c r="F144" s="8"/>
+      <c r="G144" s="8" t="s">
+        <v>711</v>
+      </c>
+      <c r="H144" s="8" t="s">
+        <v>705</v>
+      </c>
+      <c r="I144" s="8" t="s">
+        <v>712</v>
+      </c>
+      <c r="J144" s="8"/>
+      <c r="K144" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="N144" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y144" s="8"/>
+      <c r="Z144" s="8"/>
+      <c r="AA144" s="8"/>
+      <c r="AB144" s="8"/>
+      <c r="AC144" s="8"/>
+      <c r="AD144" s="8"/>
+      <c r="AE144" s="8"/>
+      <c r="AF144" s="8"/>
+      <c r="AG144" s="8"/>
+    </row>
+    <row r="145" spans="1:33" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A145" s="8" t="s">
+        <v>713</v>
+      </c>
+      <c r="B145" s="8"/>
+      <c r="C145" s="8"/>
+      <c r="D145" s="8" t="s">
+        <v>710</v>
+      </c>
+      <c r="E145" s="8"/>
+      <c r="F145" s="8"/>
+      <c r="G145" s="8" t="s">
+        <v>714</v>
+      </c>
+      <c r="H145" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="I145" s="8" t="s">
+        <v>712</v>
+      </c>
+      <c r="J145" s="8"/>
+      <c r="K145" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="N145" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y145" s="8"/>
+      <c r="Z145" s="8"/>
+      <c r="AA145" s="8"/>
+      <c r="AB145" s="8"/>
+      <c r="AC145" s="8"/>
+      <c r="AD145" s="8"/>
+      <c r="AE145" s="8"/>
+      <c r="AF145" s="8"/>
+      <c r="AG145" s="8"/>
+    </row>
+    <row r="146" spans="1:33" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A146" s="8" t="s">
+        <v>715</v>
+      </c>
+      <c r="B146" s="8"/>
+      <c r="C146" s="8"/>
+      <c r="D146" s="8" t="s">
+        <v>716</v>
+      </c>
+      <c r="E146" s="8"/>
+      <c r="F146" s="8"/>
+      <c r="G146" s="8" t="s">
+        <v>717</v>
+      </c>
+      <c r="H146" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="I146" s="8" t="s">
+        <v>718</v>
+      </c>
+      <c r="J146" s="8"/>
+      <c r="K146" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="N146" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y146" s="8"/>
+      <c r="Z146" s="8"/>
+      <c r="AA146" s="8"/>
+      <c r="AB146" s="8"/>
+      <c r="AC146" s="8"/>
+      <c r="AD146" s="8"/>
+      <c r="AE146" s="8"/>
+      <c r="AF146" s="8"/>
+      <c r="AG146" s="8"/>
+    </row>
+    <row r="147" spans="1:33" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A147" s="8" t="s">
+        <v>719</v>
+      </c>
+      <c r="B147" s="8"/>
+      <c r="C147" s="8"/>
+      <c r="D147" s="8" t="s">
+        <v>720</v>
+      </c>
+      <c r="E147" s="8"/>
+      <c r="F147" s="8"/>
+      <c r="G147" s="8" t="s">
+        <v>721</v>
+      </c>
+      <c r="H147" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="I147" s="8" t="s">
+        <v>722</v>
+      </c>
+      <c r="J147" s="8"/>
+      <c r="K147" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="N147" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y147" s="8"/>
+      <c r="Z147" s="8"/>
+      <c r="AA147" s="8"/>
+      <c r="AB147" s="8"/>
+      <c r="AC147" s="8"/>
+      <c r="AD147" s="8"/>
+      <c r="AE147" s="8"/>
+      <c r="AF147" s="8"/>
+      <c r="AG147" s="8"/>
+    </row>
+    <row r="148" spans="1:33" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A148" s="8" t="s">
+        <v>723</v>
+      </c>
+      <c r="B148" s="8"/>
+      <c r="C148" s="8"/>
+      <c r="D148" s="8" t="s">
+        <v>724</v>
+      </c>
+      <c r="E148" s="8"/>
+      <c r="F148" s="8"/>
+      <c r="G148" s="8" t="s">
+        <v>725</v>
+      </c>
+      <c r="H148" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="I148" s="8" t="s">
+        <v>726</v>
+      </c>
+      <c r="J148" s="8"/>
+      <c r="K148" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="N148" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y148" s="8"/>
+      <c r="Z148" s="8"/>
+      <c r="AA148" s="8"/>
+      <c r="AB148" s="8"/>
+      <c r="AC148" s="8"/>
+      <c r="AD148" s="8"/>
+      <c r="AE148" s="8"/>
+      <c r="AF148" s="8"/>
+      <c r="AG148" s="8"/>
+    </row>
+    <row r="149" spans="1:33" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A149" s="8" t="s">
+        <v>727</v>
+      </c>
+      <c r="B149" s="8"/>
+      <c r="C149" s="8"/>
+      <c r="D149" s="8" t="s">
+        <v>728</v>
+      </c>
+      <c r="E149" s="8"/>
+      <c r="F149" s="8"/>
+      <c r="G149" s="8" t="s">
+        <v>729</v>
+      </c>
+      <c r="H149" s="8" t="s">
+        <v>730</v>
+      </c>
+      <c r="I149" s="8" t="s">
+        <v>731</v>
+      </c>
+      <c r="J149" s="8"/>
+      <c r="K149" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="N149" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y149" s="8"/>
+      <c r="Z149" s="8"/>
+      <c r="AA149" s="8"/>
+      <c r="AB149" s="8"/>
+      <c r="AC149" s="8"/>
+      <c r="AD149" s="8"/>
+      <c r="AE149" s="8"/>
+      <c r="AF149" s="8"/>
+      <c r="AG149" s="8"/>
+    </row>
+    <row r="150" spans="1:33" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A150" s="8" t="s">
+        <v>732</v>
+      </c>
+      <c r="B150" s="8"/>
+      <c r="C150" s="8"/>
+      <c r="D150" s="8" t="s">
+        <v>733</v>
+      </c>
+      <c r="E150" s="8"/>
+      <c r="F150" s="8"/>
+      <c r="G150" s="8" t="s">
+        <v>734</v>
+      </c>
+      <c r="H150" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="I150" s="8" t="s">
+        <v>735</v>
+      </c>
+      <c r="J150" s="8"/>
+      <c r="K150" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="N150" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y150" s="8"/>
+      <c r="Z150" s="8"/>
+      <c r="AA150" s="8"/>
+      <c r="AB150" s="8"/>
+      <c r="AC150" s="8"/>
+      <c r="AD150" s="8"/>
+      <c r="AE150" s="8"/>
+      <c r="AF150" s="8"/>
+      <c r="AG150" s="8"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:N3"/>
@@ -13006,43 +13985,43 @@
     </row>
     <row r="2" ht="75" customHeight="1" spans="1:23" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
-        <v>674</v>
+        <v>736</v>
       </c>
       <c r="B2" s="9" t="s">
         <v>251</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>675</v>
+        <v>737</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>676</v>
+        <v>738</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>677</v>
+        <v>739</v>
       </c>
       <c r="F2" s="9" t="s">
-        <v>678</v>
+        <v>740</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>679</v>
+        <v>741</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>680</v>
+        <v>742</v>
       </c>
       <c r="I2" s="9" t="s">
-        <v>681</v>
+        <v>743</v>
       </c>
       <c r="J2" s="9" t="s">
         <v>95</v>
       </c>
       <c r="K2" s="9" t="s">
-        <v>682</v>
+        <v>744</v>
       </c>
       <c r="L2" s="9" t="s">
         <v>139</v>
       </c>
       <c r="M2" s="9" t="s">
-        <v>683</v>
+        <v>745</v>
       </c>
       <c r="N2" s="9" t="s">
         <v>67</v>
@@ -13051,31 +14030,31 @@
     </row>
     <row r="3" ht="45" customHeight="1" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>684</v>
+        <v>746</v>
       </c>
       <c r="B3" s="9" t="s">
         <v>251</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>675</v>
+        <v>737</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>685</v>
+        <v>747</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>686</v>
+        <v>748</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>678</v>
+        <v>740</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>687</v>
+        <v>749</v>
       </c>
       <c r="H3" s="9" t="s">
         <v>64</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>688</v>
+        <v>750</v>
       </c>
       <c r="J3" s="9" t="s">
         <v>122</v>
@@ -13111,10 +14090,10 @@
         <v>66</v>
       </c>
       <c r="U3" s="9" t="s">
-        <v>689</v>
+        <v>751</v>
       </c>
       <c r="V3" s="9" t="s">
-        <v>690</v>
+        <v>752</v>
       </c>
       <c r="W3" s="9" t="s">
         <v>70</v>
@@ -13125,7 +14104,7 @@
     </row>
     <row r="4" ht="60" customHeight="1" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>691</v>
+        <v>753</v>
       </c>
       <c r="B4" s="9" t="s">
         <v>251</v>
@@ -13134,28 +14113,28 @@
         <v>81</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>692</v>
+        <v>754</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>693</v>
+        <v>755</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>678</v>
+        <v>740</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>694</v>
+        <v>756</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>695</v>
+        <v>757</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>696</v>
+        <v>758</v>
       </c>
       <c r="J4" s="9" t="s">
         <v>95</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>697</v>
+        <v>759</v>
       </c>
       <c r="L4" s="9" t="s">
         <v>63</v>
@@ -13185,10 +14164,10 @@
         <v>66</v>
       </c>
       <c r="U4" s="9" t="s">
-        <v>689</v>
+        <v>751</v>
       </c>
       <c r="V4" s="9" t="s">
-        <v>698</v>
+        <v>760</v>
       </c>
       <c r="W4" s="9" t="s">
         <v>70</v>
@@ -13199,7 +14178,7 @@
     </row>
     <row r="5" ht="60" customHeight="1" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>699</v>
+        <v>761</v>
       </c>
       <c r="B5" s="9" t="s">
         <v>251</v>
@@ -13208,34 +14187,34 @@
         <v>81</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>700</v>
+        <v>762</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>701</v>
+        <v>763</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>678</v>
+        <v>740</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>702</v>
+        <v>764</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>703</v>
+        <v>765</v>
       </c>
       <c r="I5" s="9" t="s">
-        <v>704</v>
+        <v>766</v>
       </c>
       <c r="J5" s="9" t="s">
         <v>95</v>
       </c>
       <c r="K5" s="9" t="s">
-        <v>697</v>
+        <v>759</v>
       </c>
       <c r="L5" s="9" t="s">
         <v>63</v>
       </c>
       <c r="M5" s="9" t="s">
-        <v>705</v>
+        <v>767</v>
       </c>
       <c r="N5" s="9" t="s">
         <v>65</v>
@@ -13259,10 +14238,10 @@
         <v>66</v>
       </c>
       <c r="U5" s="9" t="s">
-        <v>689</v>
+        <v>751</v>
       </c>
       <c r="V5" s="9" t="s">
-        <v>706</v>
+        <v>768</v>
       </c>
       <c r="W5" s="9" t="s">
         <v>70</v>
@@ -13273,7 +14252,7 @@
     </row>
     <row r="6" ht="75" customHeight="1" spans="1:23" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>707</v>
+        <v>769</v>
       </c>
       <c r="B6" s="9" t="s">
         <v>251</v>
@@ -13282,34 +14261,34 @@
         <v>81</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>708</v>
+        <v>770</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>709</v>
+        <v>771</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>678</v>
+        <v>740</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>710</v>
+        <v>772</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>711</v>
+        <v>773</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>712</v>
+        <v>774</v>
       </c>
       <c r="J6" s="9" t="s">
         <v>122</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>713</v>
+        <v>775</v>
       </c>
       <c r="L6" s="9" t="s">
         <v>139</v>
       </c>
       <c r="M6" s="9" t="s">
-        <v>714</v>
+        <v>776</v>
       </c>
       <c r="N6" s="9" t="s">
         <v>67</v>
@@ -13318,31 +14297,31 @@
     </row>
     <row r="7" ht="45" customHeight="1" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>715</v>
+        <v>777</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>251</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>675</v>
+        <v>737</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>716</v>
+        <v>778</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>717</v>
+        <v>779</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>678</v>
+        <v>740</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>718</v>
+        <v>780</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>719</v>
+        <v>781</v>
       </c>
       <c r="I7" s="9" t="s">
-        <v>720</v>
+        <v>782</v>
       </c>
       <c r="J7" s="9" t="s">
         <v>122</v>
@@ -13378,10 +14357,10 @@
         <v>66</v>
       </c>
       <c r="U7" s="9" t="s">
-        <v>689</v>
+        <v>751</v>
       </c>
       <c r="V7" s="9" t="s">
-        <v>721</v>
+        <v>783</v>
       </c>
       <c r="W7" s="9" t="s">
         <v>70</v>
@@ -13392,7 +14371,7 @@
     </row>
     <row r="8" ht="78.75" customHeight="1" spans="1:24" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>722</v>
+        <v>784</v>
       </c>
       <c r="B8" s="9" t="s">
         <v>251</v>
@@ -13401,34 +14380,34 @@
         <v>116</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>723</v>
+        <v>785</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>724</v>
+        <v>786</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>678</v>
+        <v>740</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>725</v>
+        <v>787</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>726</v>
+        <v>788</v>
       </c>
       <c r="I8" s="9" t="s">
-        <v>727</v>
+        <v>789</v>
       </c>
       <c r="J8" s="9" t="s">
-        <v>728</v>
+        <v>790</v>
       </c>
       <c r="K8" s="9" t="s">
-        <v>729</v>
+        <v>791</v>
       </c>
       <c r="L8" s="9" t="s">
         <v>139</v>
       </c>
       <c r="M8" s="9" t="s">
-        <v>730</v>
+        <v>792</v>
       </c>
       <c r="N8" s="9" t="s">
         <v>65</v>
@@ -13440,7 +14419,7 @@
         <v>25.05</v>
       </c>
       <c r="Q8" s="9" t="s">
-        <v>731</v>
+        <v>793</v>
       </c>
       <c r="R8" s="9" t="s">
         <v>266</v>
@@ -13452,10 +14431,10 @@
         <v>140</v>
       </c>
       <c r="U8" s="9" t="s">
-        <v>689</v>
+        <v>751</v>
       </c>
       <c r="V8" s="9" t="s">
-        <v>732</v>
+        <v>794</v>
       </c>
       <c r="W8" s="9" t="s">
         <v>70</v>
@@ -13466,7 +14445,7 @@
     </row>
     <row r="9" ht="60" customHeight="1" spans="1:23" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>733</v>
+        <v>795</v>
       </c>
       <c r="B9" s="9" t="s">
         <v>251</v>
@@ -13475,22 +14454,22 @@
         <v>81</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>734</v>
+        <v>796</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>735</v>
+        <v>797</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>736</v>
+        <v>798</v>
       </c>
       <c r="G9" s="9" t="s">
-        <v>737</v>
+        <v>799</v>
       </c>
       <c r="H9" s="9" t="s">
-        <v>738</v>
+        <v>800</v>
       </c>
       <c r="I9" s="9" t="s">
-        <v>739</v>
+        <v>801</v>
       </c>
       <c r="J9" s="9" t="s">
         <v>122</v>
@@ -13502,7 +14481,7 @@
         <v>154</v>
       </c>
       <c r="M9" s="9" t="s">
-        <v>740</v>
+        <v>802</v>
       </c>
       <c r="N9" s="9" t="s">
         <v>67</v>
@@ -13517,25 +14496,25 @@
         <v>251</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>741</v>
+        <v>803</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>742</v>
+        <v>804</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>743</v>
+        <v>805</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>678</v>
+        <v>740</v>
       </c>
       <c r="G10" s="9" t="s">
-        <v>744</v>
+        <v>806</v>
       </c>
       <c r="H10" s="9" t="s">
         <v>64</v>
       </c>
       <c r="I10" s="9" t="s">
-        <v>745</v>
+        <v>807</v>
       </c>
       <c r="J10" s="9" t="s">
         <v>122</v>
@@ -13555,31 +14534,31 @@
     </row>
     <row r="11" spans="1:26" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>746</v>
+        <v>808</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>675</v>
+        <v>737</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>675</v>
+        <v>737</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>747</v>
+        <v>809</v>
       </c>
       <c r="G11" s="9" t="s">
-        <v>748</v>
+        <v>810</v>
       </c>
       <c r="H11" s="9" t="s">
-        <v>719</v>
+        <v>781</v>
       </c>
       <c r="I11" s="9" t="s">
-        <v>749</v>
+        <v>811</v>
       </c>
       <c r="J11" s="9" t="s">
         <v>95</v>
       </c>
       <c r="K11" s="9" t="s">
-        <v>750</v>
+        <v>812</v>
       </c>
       <c r="L11" s="8" t="s">
         <v>154</v>
@@ -13659,7 +14638,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:23" s="13" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
-        <v>751</v>
+        <v>813</v>
       </c>
       <c r="B1" s="13" t="s">
         <v>20</v>
@@ -13668,16 +14647,16 @@
         <v>21</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>752</v>
+        <v>814</v>
       </c>
       <c r="E1" s="13" t="s">
-        <v>753</v>
+        <v>815</v>
       </c>
       <c r="F1" s="13" t="s">
         <v>26</v>
       </c>
       <c r="G1" s="13" t="s">
-        <v>754</v>
+        <v>816</v>
       </c>
       <c r="H1" s="13" t="s">
         <v>43</v>
@@ -13686,7 +14665,7 @@
         <v>44</v>
       </c>
       <c r="J1" s="13" t="s">
-        <v>755</v>
+        <v>817</v>
       </c>
       <c r="K1" s="13" t="s">
         <v>29</v>
@@ -13695,7 +14674,7 @@
         <v>32</v>
       </c>
       <c r="M1" s="13" t="s">
-        <v>756</v>
+        <v>818</v>
       </c>
       <c r="N1" s="13" t="s">
         <v>33</v>
@@ -13730,7 +14709,7 @@
     </row>
     <row r="2" ht="60" customHeight="1" spans="1:23" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
-        <v>757</v>
+        <v>819</v>
       </c>
       <c r="B2" s="9" t="s">
         <v>53</v>
@@ -13739,16 +14718,16 @@
         <v>81</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>758</v>
+        <v>820</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>759</v>
+        <v>821</v>
       </c>
       <c r="F2" s="9" t="s">
         <v>129</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>760</v>
+        <v>822</v>
       </c>
       <c r="H2" s="9" t="s">
         <v>133</v>
@@ -13760,7 +14739,7 @@
         <v>95</v>
       </c>
       <c r="K2" s="9" t="s">
-        <v>761</v>
+        <v>823</v>
       </c>
       <c r="L2" s="9" t="s">
         <v>65</v>
@@ -13790,7 +14769,7 @@
         <v>109</v>
       </c>
       <c r="U2" s="9" t="s">
-        <v>762</v>
+        <v>824</v>
       </c>
       <c r="V2" s="9" t="s">
         <v>70</v>
@@ -13801,7 +14780,7 @@
     </row>
     <row r="3" ht="60" customHeight="1" spans="1:23" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>763</v>
+        <v>825</v>
       </c>
       <c r="B3" s="9" t="s">
         <v>53</v>
@@ -13810,16 +14789,16 @@
         <v>81</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>764</v>
+        <v>826</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>759</v>
+        <v>821</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>765</v>
+        <v>827</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>766</v>
+        <v>828</v>
       </c>
       <c r="H3" s="9" t="s">
         <v>133</v>
@@ -13831,7 +14810,7 @@
         <v>95</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>761</v>
+        <v>823</v>
       </c>
       <c r="L3" s="9" t="s">
         <v>65</v>
@@ -13861,7 +14840,7 @@
         <v>109</v>
       </c>
       <c r="U3" s="9" t="s">
-        <v>767</v>
+        <v>829</v>
       </c>
       <c r="V3" s="9" t="s">
         <v>70</v>
@@ -13872,7 +14851,7 @@
     </row>
     <row r="4" ht="60" customHeight="1" spans="1:23" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>768</v>
+        <v>830</v>
       </c>
       <c r="B4" s="9" t="s">
         <v>53</v>
@@ -13881,16 +14860,16 @@
         <v>81</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>769</v>
+        <v>831</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>759</v>
+        <v>821</v>
       </c>
       <c r="F4" s="9" t="s">
         <v>137</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>766</v>
+        <v>828</v>
       </c>
       <c r="H4" s="9" t="s">
         <v>133</v>
@@ -13902,7 +14881,7 @@
         <v>122</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>761</v>
+        <v>823</v>
       </c>
       <c r="L4" s="9" t="s">
         <v>65</v>
@@ -13932,7 +14911,7 @@
         <v>109</v>
       </c>
       <c r="U4" s="9" t="s">
-        <v>770</v>
+        <v>832</v>
       </c>
       <c r="V4" s="9" t="s">
         <v>70</v>
@@ -13943,7 +14922,7 @@
     </row>
     <row r="5" ht="60" customHeight="1" spans="1:23" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>771</v>
+        <v>833</v>
       </c>
       <c r="B5" s="9" t="s">
         <v>53</v>
@@ -13952,16 +14931,16 @@
         <v>81</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>772</v>
+        <v>834</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>759</v>
+        <v>821</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>773</v>
+        <v>835</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>774</v>
+        <v>836</v>
       </c>
       <c r="H5" s="9" t="s">
         <v>133</v>
@@ -13973,7 +14952,7 @@
         <v>95</v>
       </c>
       <c r="K5" s="9" t="s">
-        <v>761</v>
+        <v>823</v>
       </c>
       <c r="L5" s="9" t="s">
         <v>65</v>
@@ -14003,7 +14982,7 @@
         <v>109</v>
       </c>
       <c r="U5" s="9" t="s">
-        <v>775</v>
+        <v>837</v>
       </c>
       <c r="V5" s="9" t="s">
         <v>70</v>
@@ -14014,7 +14993,7 @@
     </row>
     <row r="6" ht="60" customHeight="1" spans="1:23" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>776</v>
+        <v>838</v>
       </c>
       <c r="B6" s="9" t="s">
         <v>53</v>
@@ -14023,22 +15002,22 @@
         <v>81</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>777</v>
+        <v>839</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>759</v>
+        <v>821</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>778</v>
+        <v>840</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>779</v>
+        <v>841</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>780</v>
+        <v>842</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>781</v>
+        <v>843</v>
       </c>
       <c r="J6" s="9" t="s">
         <v>95</v>
@@ -14074,7 +15053,7 @@
         <v>109</v>
       </c>
       <c r="U6" s="9" t="s">
-        <v>782</v>
+        <v>844</v>
       </c>
       <c r="V6" s="9" t="s">
         <v>70</v>
@@ -14085,7 +15064,7 @@
     </row>
     <row r="7" ht="60" customHeight="1" spans="1:23" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>783</v>
+        <v>845</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>53</v>
@@ -14094,19 +15073,19 @@
         <v>81</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>784</v>
+        <v>846</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>759</v>
+        <v>821</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>785</v>
+        <v>847</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>786</v>
+        <v>848</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>780</v>
+        <v>842</v>
       </c>
       <c r="I7" s="9" t="s">
         <v>64</v>
@@ -14145,7 +15124,7 @@
         <v>109</v>
       </c>
       <c r="U7" s="9" t="s">
-        <v>787</v>
+        <v>849</v>
       </c>
       <c r="V7" s="9" t="s">
         <v>70</v>
@@ -14156,7 +15135,7 @@
     </row>
     <row r="8" ht="60" customHeight="1" spans="1:23" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>788</v>
+        <v>850</v>
       </c>
       <c r="B8" s="9" t="s">
         <v>53</v>
@@ -14165,28 +15144,28 @@
         <v>116</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>789</v>
+        <v>851</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>759</v>
+        <v>821</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>790</v>
+        <v>852</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>791</v>
+        <v>853</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>780</v>
+        <v>842</v>
       </c>
       <c r="I8" s="9" t="s">
-        <v>792</v>
+        <v>854</v>
       </c>
       <c r="J8" s="9" t="s">
         <v>122</v>
       </c>
       <c r="K8" s="9" t="s">
-        <v>793</v>
+        <v>855</v>
       </c>
       <c r="L8" s="9" t="s">
         <v>65</v>
@@ -14216,7 +15195,7 @@
         <v>109</v>
       </c>
       <c r="U8" s="9" t="s">
-        <v>794</v>
+        <v>856</v>
       </c>
       <c r="V8" s="9" t="s">
         <v>70</v>
@@ -14249,7 +15228,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AF28"/>
+  <dimension ref="A1:AF29"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -14267,7 +15246,7 @@
   <sheetData>
     <row r="1" ht="27.95" customHeight="1" spans="1:32" s="13" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
-        <v>751</v>
+        <v>813</v>
       </c>
       <c r="B1" s="13" t="s">
         <v>20</v>
@@ -14276,16 +15255,16 @@
         <v>21</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>752</v>
+        <v>814</v>
       </c>
       <c r="E1" s="13" t="s">
-        <v>753</v>
+        <v>815</v>
       </c>
       <c r="F1" s="13" t="s">
         <v>26</v>
       </c>
       <c r="G1" s="13" t="s">
-        <v>754</v>
+        <v>816</v>
       </c>
       <c r="H1" s="13" t="s">
         <v>43</v>
@@ -14294,7 +15273,7 @@
         <v>44</v>
       </c>
       <c r="J1" s="13" t="s">
-        <v>755</v>
+        <v>817</v>
       </c>
       <c r="K1" s="13" t="s">
         <v>29</v>
@@ -14303,7 +15282,7 @@
         <v>32</v>
       </c>
       <c r="M1" s="13" t="s">
-        <v>756</v>
+        <v>818</v>
       </c>
       <c r="N1" s="13" t="s">
         <v>33</v>
@@ -14365,31 +15344,31 @@
     </row>
     <row r="2" ht="120" customHeight="1" spans="1:23" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
-        <v>795</v>
+        <v>857</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>796</v>
+        <v>858</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>797</v>
+        <v>859</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>798</v>
+        <v>860</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>799</v>
+        <v>861</v>
       </c>
       <c r="F2" s="9" t="s">
-        <v>800</v>
+        <v>862</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>801</v>
+        <v>863</v>
       </c>
       <c r="J2" s="9" t="s">
         <v>61</v>
       </c>
       <c r="K2" s="9" t="s">
-        <v>802</v>
+        <v>864</v>
       </c>
       <c r="L2" s="9" t="s">
         <v>65</v>
@@ -14416,10 +15395,10 @@
         <v>66</v>
       </c>
       <c r="T2" s="8" t="s">
-        <v>803</v>
+        <v>865</v>
       </c>
       <c r="U2" s="8" t="s">
-        <v>804</v>
+        <v>866</v>
       </c>
       <c r="V2" s="9" t="s">
         <v>70</v>
@@ -14430,14 +15409,14 @@
     </row>
     <row r="3" spans="1:23" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>805</v>
+        <v>867</v>
       </c>
       <c r="B3" s="9" t="s">
         <v>53</v>
       </c>
       <c r="C3" s="9"/>
       <c r="D3" s="9" t="s">
-        <v>806</v>
+        <v>868</v>
       </c>
       <c r="E3" s="9" t="s">
         <v>297</v>
@@ -14446,7 +15425,7 @@
         <v>213</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>807</v>
+        <v>869</v>
       </c>
       <c r="H3" s="9"/>
       <c r="I3" s="9"/>
@@ -14481,10 +15460,10 @@
         <v>66</v>
       </c>
       <c r="T3" s="8" t="s">
-        <v>808</v>
+        <v>870</v>
       </c>
       <c r="U3" s="8" t="s">
-        <v>809</v>
+        <v>871</v>
       </c>
       <c r="V3" s="9" t="s">
         <v>70</v>
@@ -14495,23 +15474,23 @@
     </row>
     <row r="4" spans="1:23" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>810</v>
+        <v>872</v>
       </c>
       <c r="B4" s="9" t="s">
         <v>53</v>
       </c>
       <c r="C4" s="9"/>
       <c r="D4" s="9" t="s">
-        <v>811</v>
+        <v>873</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>812</v>
+        <v>874</v>
       </c>
       <c r="F4" s="9" t="s">
         <v>213</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>813</v>
+        <v>875</v>
       </c>
       <c r="H4" s="9"/>
       <c r="I4" s="9"/>
@@ -14560,15 +15539,15 @@
     </row>
     <row r="5" spans="1:32" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>814</v>
+        <v>876</v>
       </c>
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
       <c r="D5" s="9" t="s">
-        <v>815</v>
+        <v>877</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>816</v>
+        <v>878</v>
       </c>
       <c r="F5" s="9" t="s">
         <v>213</v>
@@ -14630,21 +15609,21 @@
     </row>
     <row r="6" spans="1:32" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>817</v>
+        <v>879</v>
       </c>
       <c r="B6" s="9"/>
       <c r="C6" s="9"/>
       <c r="D6" s="9" t="s">
-        <v>818</v>
+        <v>880</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>819</v>
+        <v>881</v>
       </c>
       <c r="F6" s="9" t="s">
         <v>213</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>820</v>
+        <v>882</v>
       </c>
       <c r="H6" s="9"/>
       <c r="I6" s="9"/>
@@ -14700,21 +15679,21 @@
     </row>
     <row r="7" spans="1:32" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>821</v>
+        <v>883</v>
       </c>
       <c r="B7" s="9"/>
       <c r="C7" s="9"/>
       <c r="D7" s="9" t="s">
-        <v>822</v>
+        <v>884</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>823</v>
+        <v>885</v>
       </c>
       <c r="F7" s="9" t="s">
         <v>213</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>824</v>
+        <v>886</v>
       </c>
       <c r="H7" s="9"/>
       <c r="I7" s="9"/>
@@ -14770,7 +15749,7 @@
     </row>
     <row r="8" spans="1:32" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>825</v>
+        <v>887</v>
       </c>
       <c r="B8" s="9"/>
       <c r="C8" s="9"/>
@@ -14778,7 +15757,7 @@
         <v>421</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>826</v>
+        <v>888</v>
       </c>
       <c r="F8" s="9" t="s">
         <v>213</v>
@@ -14817,10 +15796,10 @@
         <v>66</v>
       </c>
       <c r="T8" s="8" t="s">
-        <v>827</v>
+        <v>889</v>
       </c>
       <c r="U8" s="8" t="s">
-        <v>828</v>
+        <v>890</v>
       </c>
       <c r="V8" s="9" t="s">
         <v>70</v>
@@ -14840,7 +15819,7 @@
     </row>
     <row r="9" spans="1:32" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>829</v>
+        <v>891</v>
       </c>
       <c r="B9" s="9"/>
       <c r="C9" s="9"/>
@@ -14910,21 +15889,21 @@
     </row>
     <row r="10" spans="1:32" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>830</v>
+        <v>892</v>
       </c>
       <c r="B10" s="9"/>
       <c r="C10" s="9"/>
       <c r="D10" s="9" t="s">
-        <v>831</v>
+        <v>893</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>832</v>
+        <v>894</v>
       </c>
       <c r="F10" s="9" t="s">
         <v>213</v>
       </c>
       <c r="G10" s="9" t="s">
-        <v>833</v>
+        <v>895</v>
       </c>
       <c r="H10" s="9"/>
       <c r="I10" s="9"/>
@@ -14957,10 +15936,10 @@
         <v>66</v>
       </c>
       <c r="T10" s="8" t="s">
-        <v>834</v>
+        <v>896</v>
       </c>
       <c r="U10" s="8" t="s">
-        <v>835</v>
+        <v>897</v>
       </c>
       <c r="V10" s="9" t="s">
         <v>70</v>
@@ -14980,21 +15959,21 @@
     </row>
     <row r="11" spans="1:32" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>836</v>
+        <v>898</v>
       </c>
       <c r="B11" s="9"/>
       <c r="C11" s="9"/>
       <c r="D11" s="9" t="s">
-        <v>837</v>
+        <v>899</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>838</v>
+        <v>900</v>
       </c>
       <c r="F11" s="9" t="s">
         <v>213</v>
       </c>
       <c r="G11" s="9" t="s">
-        <v>839</v>
+        <v>901</v>
       </c>
       <c r="H11" s="9"/>
       <c r="I11" s="9"/>
@@ -15027,10 +16006,10 @@
         <v>66</v>
       </c>
       <c r="T11" s="8" t="s">
-        <v>840</v>
+        <v>902</v>
       </c>
       <c r="U11" s="8" t="s">
-        <v>841</v>
+        <v>903</v>
       </c>
       <c r="V11" s="9" t="s">
         <v>70</v>
@@ -15050,7 +16029,7 @@
     </row>
     <row r="12" spans="1:32" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>842</v>
+        <v>904</v>
       </c>
       <c r="B12" s="9"/>
       <c r="C12" s="9"/>
@@ -15058,7 +16037,7 @@
         <v>574</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>843</v>
+        <v>905</v>
       </c>
       <c r="F12" s="9" t="s">
         <v>213</v>
@@ -15120,21 +16099,21 @@
     </row>
     <row r="13" spans="1:32" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
-        <v>844</v>
+        <v>906</v>
       </c>
       <c r="B13" s="9"/>
       <c r="C13" s="9"/>
       <c r="D13" s="9" t="s">
-        <v>845</v>
+        <v>907</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>846</v>
+        <v>908</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>213</v>
       </c>
       <c r="G13" s="9" t="s">
-        <v>847</v>
+        <v>909</v>
       </c>
       <c r="H13" s="9"/>
       <c r="I13" s="9"/>
@@ -15167,10 +16146,10 @@
         <v>66</v>
       </c>
       <c r="T13" s="8" t="s">
-        <v>848</v>
+        <v>910</v>
       </c>
       <c r="U13" s="8" t="s">
-        <v>849</v>
+        <v>911</v>
       </c>
       <c r="V13" s="9" t="s">
         <v>70</v>
@@ -15190,7 +16169,7 @@
     </row>
     <row r="14" spans="1:32" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
-        <v>850</v>
+        <v>912</v>
       </c>
       <c r="B14" s="9"/>
       <c r="C14" s="9"/>
@@ -15204,7 +16183,7 @@
         <v>213</v>
       </c>
       <c r="G14" s="9" t="s">
-        <v>851</v>
+        <v>913</v>
       </c>
       <c r="H14" s="9"/>
       <c r="I14" s="9"/>
@@ -15260,23 +16239,23 @@
     </row>
     <row r="15" spans="1:32" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>852</v>
+        <v>914</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>796</v>
+        <v>858</v>
       </c>
       <c r="C15" s="9"/>
       <c r="D15" s="9" t="s">
-        <v>853</v>
+        <v>915</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>854</v>
+        <v>916</v>
       </c>
       <c r="F15" s="9" t="s">
         <v>213</v>
       </c>
       <c r="G15" s="9" t="s">
-        <v>855</v>
+        <v>917</v>
       </c>
       <c r="H15" s="9"/>
       <c r="I15" s="9"/>
@@ -15309,10 +16288,10 @@
         <v>66</v>
       </c>
       <c r="T15" s="8" t="s">
-        <v>856</v>
+        <v>918</v>
       </c>
       <c r="U15" s="8" t="s">
-        <v>857</v>
+        <v>919</v>
       </c>
       <c r="V15" s="9" t="s">
         <v>70</v>
@@ -15332,10 +16311,10 @@
     </row>
     <row r="16" spans="1:32" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
+        <v>920</v>
+      </c>
+      <c r="B16" s="9" t="s">
         <v>858</v>
-      </c>
-      <c r="B16" s="9" t="s">
-        <v>796</v>
       </c>
       <c r="C16" s="9"/>
       <c r="D16" s="9" t="s">
@@ -15404,23 +16383,23 @@
     </row>
     <row r="17" spans="1:32" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
-        <v>859</v>
+        <v>921</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>796</v>
+        <v>858</v>
       </c>
       <c r="C17" s="9"/>
       <c r="D17" s="9" t="s">
-        <v>853</v>
+        <v>915</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>860</v>
+        <v>922</v>
       </c>
       <c r="F17" s="9" t="s">
         <v>213</v>
       </c>
       <c r="G17" s="9" t="s">
-        <v>861</v>
+        <v>923</v>
       </c>
       <c r="H17" s="9"/>
       <c r="I17" s="9"/>
@@ -15455,10 +16434,10 @@
         <v>66</v>
       </c>
       <c r="T17" s="8" t="s">
-        <v>862</v>
+        <v>924</v>
       </c>
       <c r="U17" s="8" t="s">
-        <v>863</v>
+        <v>925</v>
       </c>
       <c r="V17" s="9" t="s">
         <v>70</v>
@@ -15478,23 +16457,23 @@
     </row>
     <row r="18" spans="1:32" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
-        <v>864</v>
+        <v>926</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>796</v>
+        <v>858</v>
       </c>
       <c r="C18" s="9"/>
       <c r="D18" s="9" t="s">
-        <v>865</v>
+        <v>927</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>866</v>
+        <v>928</v>
       </c>
       <c r="F18" s="9" t="s">
         <v>213</v>
       </c>
       <c r="G18" s="9" t="s">
-        <v>867</v>
+        <v>929</v>
       </c>
       <c r="H18" s="9"/>
       <c r="I18" s="9"/>
@@ -15529,10 +16508,10 @@
         <v>66</v>
       </c>
       <c r="T18" s="8" t="s">
-        <v>868</v>
+        <v>930</v>
       </c>
       <c r="U18" s="8" t="s">
-        <v>869</v>
+        <v>931</v>
       </c>
       <c r="V18" s="9" t="s">
         <v>70</v>
@@ -15552,23 +16531,23 @@
     </row>
     <row r="19" spans="1:32" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
-        <v>870</v>
+        <v>932</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>796</v>
+        <v>858</v>
       </c>
       <c r="C19" s="9"/>
       <c r="D19" s="9" t="s">
-        <v>871</v>
+        <v>933</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>872</v>
+        <v>934</v>
       </c>
       <c r="F19" s="9" t="s">
         <v>213</v>
       </c>
       <c r="G19" s="9" t="s">
-        <v>873</v>
+        <v>935</v>
       </c>
       <c r="H19" s="9"/>
       <c r="I19" s="9"/>
@@ -15603,10 +16582,10 @@
         <v>66</v>
       </c>
       <c r="T19" s="8" t="s">
-        <v>874</v>
+        <v>936</v>
       </c>
       <c r="U19" s="8" t="s">
-        <v>875</v>
+        <v>937</v>
       </c>
       <c r="V19" s="9" t="s">
         <v>70</v>
@@ -15626,23 +16605,23 @@
     </row>
     <row r="20" spans="1:32" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
-        <v>876</v>
+        <v>938</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>796</v>
+        <v>858</v>
       </c>
       <c r="C20" s="9"/>
       <c r="D20" s="9" t="s">
-        <v>871</v>
+        <v>933</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>877</v>
+        <v>939</v>
       </c>
       <c r="F20" s="9" t="s">
         <v>213</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>878</v>
+        <v>940</v>
       </c>
       <c r="H20" s="9"/>
       <c r="I20" s="9"/>
@@ -15677,10 +16656,10 @@
         <v>66</v>
       </c>
       <c r="T20" s="8" t="s">
-        <v>879</v>
+        <v>941</v>
       </c>
       <c r="U20" s="8" t="s">
-        <v>880</v>
+        <v>942</v>
       </c>
       <c r="V20" s="9" t="s">
         <v>70</v>
@@ -15700,7 +16679,7 @@
     </row>
     <row r="21" spans="1:32" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
-        <v>881</v>
+        <v>943</v>
       </c>
       <c r="B21" s="9"/>
       <c r="C21" s="9"/>
@@ -15708,7 +16687,7 @@
         <v>430</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>882</v>
+        <v>944</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>213</v>
@@ -15770,15 +16749,15 @@
     </row>
     <row r="22" spans="1:32" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
-        <v>883</v>
+        <v>945</v>
       </c>
       <c r="B22" s="9"/>
       <c r="C22" s="9"/>
       <c r="D22" s="9" t="s">
-        <v>884</v>
+        <v>946</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>885</v>
+        <v>947</v>
       </c>
       <c r="F22" s="9" t="s">
         <v>213</v>
@@ -15840,7 +16819,7 @@
     </row>
     <row r="23" spans="1:32" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
-        <v>886</v>
+        <v>948</v>
       </c>
       <c r="B23" s="9"/>
       <c r="C23" s="9"/>
@@ -15854,7 +16833,7 @@
         <v>213</v>
       </c>
       <c r="G23" s="9" t="s">
-        <v>887</v>
+        <v>949</v>
       </c>
       <c r="H23" s="9"/>
       <c r="I23" s="9"/>
@@ -15910,7 +16889,7 @@
     </row>
     <row r="24" spans="1:32" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
-        <v>888</v>
+        <v>950</v>
       </c>
       <c r="B24" s="9"/>
       <c r="C24" s="9"/>
@@ -15918,7 +16897,7 @@
         <v>600</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>889</v>
+        <v>951</v>
       </c>
       <c r="F24" s="9" t="s">
         <v>213</v>
@@ -15980,21 +16959,21 @@
     </row>
     <row r="25" spans="1:32" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">
-        <v>890</v>
+        <v>952</v>
       </c>
       <c r="B25" s="9"/>
       <c r="C25" s="9"/>
       <c r="D25" s="9" t="s">
-        <v>891</v>
+        <v>953</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>892</v>
+        <v>954</v>
       </c>
       <c r="F25" s="9" t="s">
         <v>213</v>
       </c>
       <c r="G25" s="9" t="s">
-        <v>893</v>
+        <v>955</v>
       </c>
       <c r="H25" s="9"/>
       <c r="I25" s="9"/>
@@ -16050,7 +17029,7 @@
     </row>
     <row r="26" spans="1:32" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="9" t="s">
-        <v>894</v>
+        <v>956</v>
       </c>
       <c r="B26" s="9"/>
       <c r="C26" s="9"/>
@@ -16058,7 +17037,7 @@
         <v>444</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>895</v>
+        <v>957</v>
       </c>
       <c r="F26" s="9" t="s">
         <v>213</v>
@@ -16097,10 +17076,10 @@
         <v>66</v>
       </c>
       <c r="T26" s="8" t="s">
-        <v>896</v>
+        <v>958</v>
       </c>
       <c r="U26" s="8" t="s">
-        <v>897</v>
+        <v>959</v>
       </c>
       <c r="V26" s="9" t="s">
         <v>70</v>
@@ -16120,12 +17099,12 @@
     </row>
     <row r="27" spans="1:32" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="9" t="s">
-        <v>898</v>
+        <v>960</v>
       </c>
       <c r="B27" s="9"/>
       <c r="C27" s="9"/>
       <c r="D27" s="9" t="s">
-        <v>899</v>
+        <v>961</v>
       </c>
       <c r="E27" s="9" t="s">
         <v>589</v>
@@ -16167,10 +17146,10 @@
         <v>66</v>
       </c>
       <c r="T27" s="8" t="s">
-        <v>900</v>
+        <v>962</v>
       </c>
       <c r="U27" s="8" t="s">
-        <v>901</v>
+        <v>963</v>
       </c>
       <c r="V27" s="9" t="s">
         <v>70</v>
@@ -16190,23 +17169,23 @@
     </row>
     <row r="28" spans="1:32" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="8" t="s">
-        <v>902</v>
+        <v>964</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>796</v>
+        <v>858</v>
       </c>
       <c r="C28" s="8"/>
       <c r="D28" s="8" t="s">
         <v>671</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>903</v>
+        <v>965</v>
       </c>
       <c r="F28" s="8" t="s">
         <v>213</v>
       </c>
       <c r="G28" s="8" t="s">
-        <v>904</v>
+        <v>966</v>
       </c>
       <c r="H28" s="8"/>
       <c r="I28" s="8"/>
@@ -16228,6 +17207,47 @@
       <c r="AD28" s="8"/>
       <c r="AE28" s="8"/>
       <c r="AF28" s="8"/>
+    </row>
+    <row r="29" spans="1:32" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="8" t="s">
+        <v>967</v>
+      </c>
+      <c r="B29" s="8" t="s">
+        <v>858</v>
+      </c>
+      <c r="C29" s="8"/>
+      <c r="D29" s="8" t="s">
+        <v>968</v>
+      </c>
+      <c r="E29" s="8" t="s">
+        <v>969</v>
+      </c>
+      <c r="F29" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="G29" s="8" t="s">
+        <v>970</v>
+      </c>
+      <c r="H29" s="8"/>
+      <c r="I29" s="8"/>
+      <c r="J29" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="K29" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="L29" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="X29" s="8"/>
+      <c r="Y29" s="8"/>
+      <c r="Z29" s="8"/>
+      <c r="AA29" s="8"/>
+      <c r="AB29" s="8"/>
+      <c r="AC29" s="8"/>
+      <c r="AD29" s="8"/>
+      <c r="AE29" s="8"/>
+      <c r="AF29" s="8"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>